<commit_message>
Skipperplan: 09.05.2026 20:05 UTC
</commit_message>
<xml_diff>
--- a/skipperplan.xlsx
+++ b/skipperplan.xlsx
@@ -26069,7 +26069,7 @@
         <v>7</v>
       </c>
       <c r="J212" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K212" s="3" t="s">
         <v>34</v>
@@ -54525,7 +54525,7 @@
         <v>8</v>
       </c>
       <c r="J575" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K575" s="5" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Skipperplan: 09.05.2026 23:09 UTC
</commit_message>
<xml_diff>
--- a/skipperplan.xlsx
+++ b/skipperplan.xlsx
@@ -24233,82 +24233,82 @@
       </c>
     </row>
     <row r="189" spans="1:26">
-      <c r="A189" s="6" t="s">
+      <c r="A189" s="7" t="s">
         <v>545</v>
       </c>
-      <c r="B189" s="6" t="s">
+      <c r="B189" s="7" t="s">
         <v>565</v>
       </c>
-      <c r="C189" s="6" t="s">
+      <c r="C189" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D189" s="6" t="s">
+      <c r="D189" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E189" s="6" t="s">
+      <c r="E189" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F189" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G189" s="6" t="s">
+      <c r="F189" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G189" s="7" t="s">
         <v>776</v>
       </c>
-      <c r="H189" s="6" t="s">
+      <c r="H189" s="7" t="s">
         <v>777</v>
       </c>
-      <c r="I189" s="6">
+      <c r="I189" s="7">
         <v>9</v>
       </c>
-      <c r="J189" s="6">
-        <v>0</v>
-      </c>
-      <c r="K189" s="6" t="s">
+      <c r="J189" s="7">
+        <v>2</v>
+      </c>
+      <c r="K189" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="L189" s="6" t="s">
+      <c r="L189" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="M189" s="6" t="s">
+      <c r="M189" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="N189" s="6" t="s">
+      <c r="N189" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="O189" s="6" t="s">
+      <c r="O189" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="P189" s="6" t="s">
+      <c r="P189" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="Q189" s="6" t="s">
+      <c r="Q189" s="7" t="s">
         <v>773</v>
       </c>
-      <c r="R189" s="6" t="s">
+      <c r="R189" s="7" t="s">
         <v>778</v>
       </c>
-      <c r="S189" s="6" t="s">
+      <c r="S189" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="T189" s="6" t="s">
+      <c r="T189" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="U189" s="6" t="s">
+      <c r="U189" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="V189" s="6">
+      <c r="V189" s="7">
         <v>2018</v>
       </c>
-      <c r="W189" s="6" t="s">
-        <v>439</v>
-      </c>
-      <c r="X189" s="6" t="s">
+      <c r="W189" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="X189" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="Y189" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="Z189" s="6"/>
+      <c r="Y189" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z189" s="7"/>
     </row>
     <row r="190" spans="1:26">
       <c r="A190" s="6" t="s">
@@ -25125,7 +25125,7 @@
         <v>9</v>
       </c>
       <c r="J200" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K200" s="3" t="s">
         <v>34</v>
@@ -28189,7 +28189,7 @@
         <v>8</v>
       </c>
       <c r="J239" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K239" s="4" t="s">
         <v>34</v>
@@ -41841,7 +41841,7 @@
         <v>8</v>
       </c>
       <c r="J413" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K413" s="5" t="s">
         <v>34</v>

</xml_diff>

<commit_message>
Skipperplan: 11.05.2026 03:01 UTC
</commit_message>
<xml_diff>
--- a/skipperplan.xlsx
+++ b/skipperplan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25743" uniqueCount="2970">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25770" uniqueCount="2972">
   <si>
     <t>Startdatum</t>
   </si>
@@ -3429,7 +3429,7 @@
     <t>15220</t>
   </si>
   <si>
-    <t>Jonas B</t>
+    <t>Jonas B, Lukas H</t>
   </si>
   <si>
     <t>Fabian F</t>
@@ -3624,7 +3624,7 @@
     <t>15726</t>
   </si>
   <si>
-    <t>Philipp K, Christian K, Florian B, Korbinian R, Sebastian W, Martin W, Marlon S, Lukas H</t>
+    <t>Philipp K, Christian K, Florian B, Korbinian R, Sebastian W, Martin W, Marlon S</t>
   </si>
   <si>
     <t>15727</t>
@@ -3849,7 +3849,7 @@
     <t>15528</t>
   </si>
   <si>
-    <t>Simon B, Lukas F, Sven H</t>
+    <t>Simon B, Lukas F, Sven H, Lukas H</t>
   </si>
   <si>
     <t>Lennart M</t>
@@ -5109,7 +5109,7 @@
     <t>15741</t>
   </si>
   <si>
-    <t>Nils K, Martin W, Marc D, Hendrik B, David S, Jaqueline N</t>
+    <t>Nils K, Martin W, Marc D, Hendrik B, Jaqueline N</t>
   </si>
   <si>
     <t>15743</t>
@@ -6039,7 +6039,7 @@
     <t>16245</t>
   </si>
   <si>
-    <t>Andreas N, David Ben T, Martin W, Matthias S, Christina T, Benjamin W, Jasper P</t>
+    <t>Andreas N, David Ben T, Martin W, Matthias S, Christina T, Benjamin W, Jasper P, Miro W</t>
   </si>
   <si>
     <t>16246</t>
@@ -8067,7 +8067,7 @@
     <t>16819</t>
   </si>
   <si>
-    <t>Nicole M, Johanna S, Miriam M, Marlon S, Leon H, Constantin R</t>
+    <t>Nicole M, Johanna S, Miriam M, Marlon S, Leon H, Constantin R, Miro W</t>
   </si>
   <si>
     <t>17159</t>
@@ -8914,6 +8914,12 @@
   </si>
   <si>
     <t>Neue Bewerbungen</t>
+  </si>
+  <si>
+    <t>Neue Bewerbung(en)</t>
+  </si>
+  <si>
+    <t>Miro W</t>
   </si>
   <si>
     <t>ID</t>
@@ -11505,7 +11511,7 @@
         <v>9</v>
       </c>
       <c r="J27" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K27" s="5" t="s">
         <v>34</v>
@@ -11661,7 +11667,7 @@
         <v>8</v>
       </c>
       <c r="J29" s="7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K29" s="7" t="s">
         <v>34</v>
@@ -12767,7 +12773,7 @@
         <v>8</v>
       </c>
       <c r="J43" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K43" s="7" t="s">
         <v>34</v>
@@ -13553,7 +13559,7 @@
         <v>10</v>
       </c>
       <c r="J53" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K53" s="5" t="s">
         <v>34</v>
@@ -13945,7 +13951,7 @@
         <v>8</v>
       </c>
       <c r="J58" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K58" s="3" t="s">
         <v>34</v>
@@ -17969,7 +17975,7 @@
         <v>9</v>
       </c>
       <c r="J109" s="5">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K109" s="5" t="s">
         <v>34</v>
@@ -18283,7 +18289,7 @@
         <v>9</v>
       </c>
       <c r="J113" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K113" s="5" t="s">
         <v>34</v>
@@ -19149,7 +19155,7 @@
         <v>9</v>
       </c>
       <c r="J124" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K124" s="3" t="s">
         <v>34</v>
@@ -22535,7 +22541,7 @@
         <v>10</v>
       </c>
       <c r="J167" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K167" s="5" t="s">
         <v>34</v>
@@ -22929,7 +22935,7 @@
         <v>8</v>
       </c>
       <c r="J172" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K172" s="3" t="s">
         <v>34</v>
@@ -23323,7 +23329,7 @@
         <v>9</v>
       </c>
       <c r="J177" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K177" s="6" t="s">
         <v>34</v>
@@ -24955,7 +24961,7 @@
         <v>51</v>
       </c>
       <c r="F198" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G198" s="3" t="s">
         <v>126</v>
@@ -25035,7 +25041,7 @@
         <v>51</v>
       </c>
       <c r="F199" s="5" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G199" s="5" t="s">
         <v>108</v>
@@ -27955,7 +27961,7 @@
         <v>8</v>
       </c>
       <c r="J236" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K236" s="3" t="s">
         <v>34</v>
@@ -28503,7 +28509,7 @@
         <v>8</v>
       </c>
       <c r="J243" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K243" s="5" t="s">
         <v>34</v>
@@ -36203,7 +36209,7 @@
         <v>8</v>
       </c>
       <c r="J341" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K341" s="5" t="s">
         <v>34</v>
@@ -36515,7 +36521,7 @@
         <v>9</v>
       </c>
       <c r="J345" s="5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K345" s="5" t="s">
         <v>34</v>
@@ -36671,7 +36677,7 @@
         <v>8</v>
       </c>
       <c r="J347" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K347" s="5" t="s">
         <v>34</v>
@@ -36817,7 +36823,7 @@
         <v>51</v>
       </c>
       <c r="F349" s="5" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G349" s="5" t="s">
         <v>929</v>
@@ -36897,7 +36903,7 @@
         <v>51</v>
       </c>
       <c r="F350" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G350" s="3" t="s">
         <v>1219</v>
@@ -36975,7 +36981,7 @@
         <v>51</v>
       </c>
       <c r="F351" s="6" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G351" s="6" t="s">
         <v>1072</v>
@@ -37053,7 +37059,7 @@
         <v>51</v>
       </c>
       <c r="F352" s="6" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G352" s="6" t="s">
         <v>866</v>
@@ -37131,7 +37137,7 @@
         <v>51</v>
       </c>
       <c r="F353" s="6" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G353" s="6" t="s">
         <v>1225</v>
@@ -37209,7 +37215,7 @@
         <v>51</v>
       </c>
       <c r="F354" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G354" s="3" t="s">
         <v>682</v>
@@ -39165,7 +39171,7 @@
         <v>51</v>
       </c>
       <c r="F379" s="5" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G379" s="5" t="s">
         <v>1143</v>
@@ -39245,7 +39251,7 @@
         <v>51</v>
       </c>
       <c r="F380" s="6" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G380" s="6" t="s">
         <v>1275</v>
@@ -39323,7 +39329,7 @@
         <v>51</v>
       </c>
       <c r="F381" s="6" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G381" s="6" t="s">
         <v>1184</v>
@@ -39401,7 +39407,7 @@
         <v>51</v>
       </c>
       <c r="F382" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G382" s="4" t="s">
         <v>287</v>
@@ -42073,7 +42079,7 @@
         <v>9</v>
       </c>
       <c r="J416" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K416" s="3" t="s">
         <v>34</v>
@@ -44575,7 +44581,7 @@
         <v>51</v>
       </c>
       <c r="F448" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G448" s="3" t="s">
         <v>108</v>
@@ -44655,7 +44661,7 @@
         <v>51</v>
       </c>
       <c r="F449" s="6" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G449" s="6" t="s">
         <v>1427</v>
@@ -44733,7 +44739,7 @@
         <v>51</v>
       </c>
       <c r="F450" s="6" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G450" s="6" t="s">
         <v>1307</v>
@@ -46541,7 +46547,7 @@
         <v>7</v>
       </c>
       <c r="J473" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K473" s="5" t="s">
         <v>34</v>
@@ -46917,7 +46923,7 @@
         <v>51</v>
       </c>
       <c r="F478" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G478" s="7" t="s">
         <v>220</v>
@@ -46997,7 +47003,7 @@
         <v>51</v>
       </c>
       <c r="F479" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G479" s="7" t="s">
         <v>929</v>
@@ -50531,7 +50537,7 @@
         <v>8</v>
       </c>
       <c r="J524" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K524" s="4" t="s">
         <v>34</v>
@@ -52877,7 +52883,7 @@
         <v>9</v>
       </c>
       <c r="J554" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K554" s="3" t="s">
         <v>34</v>
@@ -54525,7 +54531,7 @@
         <v>8</v>
       </c>
       <c r="J575" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K575" s="5" t="s">
         <v>34</v>
@@ -54759,7 +54765,7 @@
         <v>9</v>
       </c>
       <c r="J578" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K578" s="3" t="s">
         <v>34</v>
@@ -55931,7 +55937,7 @@
         <v>10</v>
       </c>
       <c r="J593" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K593" s="7" t="s">
         <v>34</v>
@@ -56241,7 +56247,7 @@
         <v>7</v>
       </c>
       <c r="J597" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K597" s="5" t="s">
         <v>34</v>
@@ -60775,7 +60781,7 @@
         <v>9</v>
       </c>
       <c r="J655" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K655" s="5" t="s">
         <v>34</v>
@@ -61399,7 +61405,7 @@
         <v>7</v>
       </c>
       <c r="J663" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K663" s="5" t="s">
         <v>34</v>
@@ -65085,7 +65091,7 @@
         <v>8</v>
       </c>
       <c r="J710" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K710" s="3" t="s">
         <v>34</v>
@@ -65385,7 +65391,7 @@
         <v>51</v>
       </c>
       <c r="F714" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G714" s="3" t="s">
         <v>1129</v>
@@ -65397,7 +65403,7 @@
         <v>9</v>
       </c>
       <c r="J714" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K714" s="3" t="s">
         <v>34</v>
@@ -65465,7 +65471,7 @@
         <v>51</v>
       </c>
       <c r="F715" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G715" s="7" t="s">
         <v>560</v>
@@ -65543,7 +65549,7 @@
         <v>51</v>
       </c>
       <c r="F716" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G716" s="7" t="s">
         <v>1858</v>
@@ -65621,7 +65627,7 @@
         <v>51</v>
       </c>
       <c r="F717" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G717" s="7" t="s">
         <v>854</v>
@@ -65699,7 +65705,7 @@
         <v>51</v>
       </c>
       <c r="F718" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G718" s="7" t="s">
         <v>1979</v>
@@ -65777,7 +65783,7 @@
         <v>51</v>
       </c>
       <c r="F719" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G719" s="4" t="s">
         <v>287</v>
@@ -65853,7 +65859,7 @@
         <v>51</v>
       </c>
       <c r="F720" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G720" s="3" t="s">
         <v>61</v>
@@ -65931,7 +65937,7 @@
         <v>51</v>
       </c>
       <c r="F721" s="5" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G721" s="5" t="s">
         <v>906</v>
@@ -66009,7 +66015,7 @@
         <v>51</v>
       </c>
       <c r="F722" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G722" s="3" t="s">
         <v>369</v>
@@ -68831,7 +68837,7 @@
         <v>51</v>
       </c>
       <c r="F758" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G758" s="7" t="s">
         <v>126</v>
@@ -68911,7 +68917,7 @@
         <v>51</v>
       </c>
       <c r="F759" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G759" s="7" t="s">
         <v>776</v>
@@ -68989,7 +68995,7 @@
         <v>51</v>
       </c>
       <c r="F760" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G760" s="7" t="s">
         <v>482</v>
@@ -69067,7 +69073,7 @@
         <v>51</v>
       </c>
       <c r="F761" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G761" s="7" t="s">
         <v>2061</v>
@@ -69145,7 +69151,7 @@
         <v>51</v>
       </c>
       <c r="F762" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G762" s="7" t="s">
         <v>352</v>
@@ -69223,7 +69229,7 @@
         <v>51</v>
       </c>
       <c r="F763" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G763" s="7" t="s">
         <v>996</v>
@@ -69313,7 +69319,7 @@
         <v>8</v>
       </c>
       <c r="J764" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K764" s="7" t="s">
         <v>34</v>
@@ -75255,7 +75261,7 @@
         <v>51</v>
       </c>
       <c r="F840" s="3" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G840" s="3" t="s">
         <v>1385</v>
@@ -75335,7 +75341,7 @@
         <v>51</v>
       </c>
       <c r="F841" s="5" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G841" s="5" t="s">
         <v>941</v>
@@ -75413,7 +75419,7 @@
         <v>51</v>
       </c>
       <c r="F842" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G842" s="7" t="s">
         <v>1858</v>
@@ -75491,7 +75497,7 @@
         <v>51</v>
       </c>
       <c r="F843" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G843" s="4" t="s">
         <v>287</v>
@@ -80353,7 +80359,7 @@
         <v>51</v>
       </c>
       <c r="F905" s="5" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G905" s="5" t="s">
         <v>256</v>
@@ -80433,7 +80439,7 @@
         <v>51</v>
       </c>
       <c r="F906" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G906" s="7" t="s">
         <v>219</v>
@@ -80511,7 +80517,7 @@
         <v>51</v>
       </c>
       <c r="F907" s="7" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G907" s="7" t="s">
         <v>2352</v>
@@ -80589,7 +80595,7 @@
         <v>51</v>
       </c>
       <c r="F908" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G908" s="4" t="s">
         <v>287</v>
@@ -80677,7 +80683,7 @@
         <v>6</v>
       </c>
       <c r="J909" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K909" s="7" t="s">
         <v>34</v>
@@ -84253,7 +84259,7 @@
         <v>1882</v>
       </c>
       <c r="F955" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G955" s="4" t="s">
         <v>287</v>
@@ -84331,7 +84337,7 @@
         <v>1882</v>
       </c>
       <c r="F956" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G956" s="4" t="s">
         <v>287</v>
@@ -86341,7 +86347,7 @@
         <v>8</v>
       </c>
       <c r="J982" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K982" s="4" t="s">
         <v>34</v>
@@ -86561,7 +86567,7 @@
         <v>30</v>
       </c>
       <c r="F985" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G985" s="4" t="s">
         <v>287</v>
@@ -86639,7 +86645,7 @@
         <v>30</v>
       </c>
       <c r="F986" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G986" s="4" t="s">
         <v>287</v>
@@ -86715,7 +86721,7 @@
         <v>30</v>
       </c>
       <c r="F987" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G987" s="4" t="s">
         <v>287</v>
@@ -86791,7 +86797,7 @@
         <v>30</v>
       </c>
       <c r="F988" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G988" s="4" t="s">
         <v>287</v>
@@ -86867,7 +86873,7 @@
         <v>30</v>
       </c>
       <c r="F989" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G989" s="4" t="s">
         <v>287</v>
@@ -91253,7 +91259,7 @@
         <v>1882</v>
       </c>
       <c r="F1046" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G1046" s="4" t="s">
         <v>287</v>
@@ -91331,7 +91337,7 @@
         <v>1882</v>
       </c>
       <c r="F1047" s="4" t="s">
-        <v>805</v>
+        <v>31</v>
       </c>
       <c r="G1047" s="4" t="s">
         <v>287</v>
@@ -98750,7 +98756,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -98789,6 +98795,104 @@
       </c>
       <c r="I1" s="1" t="s">
         <v>2962</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="3" t="s">
+        <v>2963</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>829</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="3" t="s">
+        <v>2963</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>1092</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>1102</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>1143</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="3" t="s">
+        <v>2963</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>1871</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>1887</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>853</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>2964</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="3" t="s">
+        <v>2963</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>2428</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>2649</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>2677</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>2434</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>2964</v>
       </c>
     </row>
   </sheetData>
@@ -98814,16 +98918,16 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2963</v>
+        <v>2965</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2964</v>
+        <v>2966</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2965</v>
+        <v>2967</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2966</v>
+        <v>2968</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -98840,7 +98944,7 @@
         <v>19</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -98857,7 +98961,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -98874,7 +98978,7 @@
         <v>15</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -98891,7 +98995,7 @@
         <v>14</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -98908,7 +99012,7 @@
         <v>16</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -98925,7 +99029,7 @@
         <v>14</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -98942,7 +99046,7 @@
         <v>14</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -98959,7 +99063,7 @@
         <v>13</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -98976,7 +99080,7 @@
         <v>14</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -98993,7 +99097,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -99010,7 +99114,7 @@
         <v>14</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -99027,7 +99131,7 @@
         <v>12</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -99044,7 +99148,7 @@
         <v>12</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -99061,7 +99165,7 @@
         <v>11</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -99078,7 +99182,7 @@
         <v>12</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -99095,7 +99199,7 @@
         <v>11</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -99112,7 +99216,7 @@
         <v>8</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -99129,7 +99233,7 @@
         <v>8</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -99146,7 +99250,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -99163,7 +99267,7 @@
         <v>8</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -99180,7 +99284,7 @@
         <v>8</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -99197,7 +99301,7 @@
         <v>7</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -99214,7 +99318,7 @@
         <v>7</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -99231,7 +99335,7 @@
         <v>7</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -99248,7 +99352,7 @@
         <v>7</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -99265,7 +99369,7 @@
         <v>7</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -99282,7 +99386,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -99299,7 +99403,7 @@
         <v>7</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -99316,7 +99420,7 @@
         <v>7</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -99333,7 +99437,7 @@
         <v>6</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -99350,7 +99454,7 @@
         <v>6</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -99367,7 +99471,7 @@
         <v>6</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -99384,7 +99488,7 @@
         <v>6</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -99401,7 +99505,7 @@
         <v>6</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -99418,7 +99522,7 @@
         <v>6</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -99435,7 +99539,7 @@
         <v>6</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -99452,7 +99556,7 @@
         <v>6</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>2968</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -99469,7 +99573,7 @@
         <v>5</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -99486,7 +99590,7 @@
         <v>5</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -99503,7 +99607,7 @@
         <v>5</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -99520,7 +99624,7 @@
         <v>5</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -99537,7 +99641,7 @@
         <v>5</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -99554,7 +99658,7 @@
         <v>5</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -99571,7 +99675,7 @@
         <v>5</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -99588,7 +99692,7 @@
         <v>5</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -99605,7 +99709,7 @@
         <v>5</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -99622,7 +99726,7 @@
         <v>5</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -99639,7 +99743,7 @@
         <v>7</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -99656,7 +99760,7 @@
         <v>5</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -99673,7 +99777,7 @@
         <v>5</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -99690,7 +99794,7 @@
         <v>5</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -99707,7 +99811,7 @@
         <v>5</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -99724,7 +99828,7 @@
         <v>5</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -99741,7 +99845,7 @@
         <v>5</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -99758,7 +99862,7 @@
         <v>5</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -99775,7 +99879,7 @@
         <v>5</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -99792,7 +99896,7 @@
         <v>4</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -99809,7 +99913,7 @@
         <v>4</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -99826,7 +99930,7 @@
         <v>4</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -99843,7 +99947,7 @@
         <v>4</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -99860,7 +99964,7 @@
         <v>4</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -99877,7 +99981,7 @@
         <v>4</v>
       </c>
       <c r="E63" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -99894,7 +99998,7 @@
         <v>4</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -99911,7 +100015,7 @@
         <v>4</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -99928,7 +100032,7 @@
         <v>4</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -99945,7 +100049,7 @@
         <v>4</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -99962,7 +100066,7 @@
         <v>4</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -99979,7 +100083,7 @@
         <v>4</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -99996,7 +100100,7 @@
         <v>4</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -100013,7 +100117,7 @@
         <v>4</v>
       </c>
       <c r="E71" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -100030,7 +100134,7 @@
         <v>4</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -100047,7 +100151,7 @@
         <v>4</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -100064,7 +100168,7 @@
         <v>4</v>
       </c>
       <c r="E74" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -100081,7 +100185,7 @@
         <v>5</v>
       </c>
       <c r="E75" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -100098,7 +100202,7 @@
         <v>4</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -100115,7 +100219,7 @@
         <v>4</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -100132,7 +100236,7 @@
         <v>4</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -100149,7 +100253,7 @@
         <v>4</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -100166,7 +100270,7 @@
         <v>4</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -100183,7 +100287,7 @@
         <v>4</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -100200,7 +100304,7 @@
         <v>4</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -100217,7 +100321,7 @@
         <v>4</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -100234,7 +100338,7 @@
         <v>4</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -100251,7 +100355,7 @@
         <v>6</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -100268,7 +100372,7 @@
         <v>4</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -100285,7 +100389,7 @@
         <v>3</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -100302,7 +100406,7 @@
         <v>3</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -100319,7 +100423,7 @@
         <v>3</v>
       </c>
       <c r="E89" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -100336,7 +100440,7 @@
         <v>3</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -100353,7 +100457,7 @@
         <v>3</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -100370,7 +100474,7 @@
         <v>3</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -100387,7 +100491,7 @@
         <v>3</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -100404,7 +100508,7 @@
         <v>3</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -100421,7 +100525,7 @@
         <v>3</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -100438,7 +100542,7 @@
         <v>3</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -100455,7 +100559,7 @@
         <v>3</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -100472,7 +100576,7 @@
         <v>3</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -100489,7 +100593,7 @@
         <v>3</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -100506,7 +100610,7 @@
         <v>3</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -100523,7 +100627,7 @@
         <v>3</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -100540,7 +100644,7 @@
         <v>3</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -100557,7 +100661,7 @@
         <v>3</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -100574,7 +100678,7 @@
         <v>3</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -100591,7 +100695,7 @@
         <v>3</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -100608,7 +100712,7 @@
         <v>3</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -100625,7 +100729,7 @@
         <v>3</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -100642,7 +100746,7 @@
         <v>3</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -100659,7 +100763,7 @@
         <v>3</v>
       </c>
       <c r="E109" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -100676,7 +100780,7 @@
         <v>3</v>
       </c>
       <c r="E110" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -100693,7 +100797,7 @@
         <v>3</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -100710,7 +100814,7 @@
         <v>3</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -100727,7 +100831,7 @@
         <v>3</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -100744,7 +100848,7 @@
         <v>3</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -100761,7 +100865,7 @@
         <v>3</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -100778,7 +100882,7 @@
         <v>3</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -100795,7 +100899,7 @@
         <v>4</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -100812,7 +100916,7 @@
         <v>3</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -100829,7 +100933,7 @@
         <v>3</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -100846,7 +100950,7 @@
         <v>3</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -100863,7 +100967,7 @@
         <v>3</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -100880,7 +100984,7 @@
         <v>3</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -100897,7 +101001,7 @@
         <v>3</v>
       </c>
       <c r="E123" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -100914,7 +101018,7 @@
         <v>3</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -100931,7 +101035,7 @@
         <v>3</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -100948,7 +101052,7 @@
         <v>2</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -100965,7 +101069,7 @@
         <v>2</v>
       </c>
       <c r="E127" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -100982,7 +101086,7 @@
         <v>3</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -100999,7 +101103,7 @@
         <v>2</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -101016,7 +101120,7 @@
         <v>2</v>
       </c>
       <c r="E130" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -101033,7 +101137,7 @@
         <v>2</v>
       </c>
       <c r="E131" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -101050,7 +101154,7 @@
         <v>2</v>
       </c>
       <c r="E132" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -101067,7 +101171,7 @@
         <v>2</v>
       </c>
       <c r="E133" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -101084,7 +101188,7 @@
         <v>2</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -101101,7 +101205,7 @@
         <v>2</v>
       </c>
       <c r="E135" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -101118,7 +101222,7 @@
         <v>2</v>
       </c>
       <c r="E136" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -101135,7 +101239,7 @@
         <v>2</v>
       </c>
       <c r="E137" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -101152,7 +101256,7 @@
         <v>2</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -101169,7 +101273,7 @@
         <v>2</v>
       </c>
       <c r="E139" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -101186,7 +101290,7 @@
         <v>2</v>
       </c>
       <c r="E140" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -101203,7 +101307,7 @@
         <v>2</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -101220,7 +101324,7 @@
         <v>2</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -101237,7 +101341,7 @@
         <v>2</v>
       </c>
       <c r="E143" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -101254,7 +101358,7 @@
         <v>2</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -101271,7 +101375,7 @@
         <v>2</v>
       </c>
       <c r="E145" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -101288,7 +101392,7 @@
         <v>2</v>
       </c>
       <c r="E146" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -101305,7 +101409,7 @@
         <v>2</v>
       </c>
       <c r="E147" s="9" t="s">
-        <v>2967</v>
+        <v>2969</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -101322,7 +101426,7 @@
         <v>2</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -101339,7 +101443,7 @@
         <v>2</v>
       </c>
       <c r="E149" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -101356,7 +101460,7 @@
         <v>2</v>
       </c>
       <c r="E150" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -101373,7 +101477,7 @@
         <v>2</v>
       </c>
       <c r="E151" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -101390,7 +101494,7 @@
         <v>2</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -101407,7 +101511,7 @@
         <v>2</v>
       </c>
       <c r="E153" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -101424,7 +101528,7 @@
         <v>2</v>
       </c>
       <c r="E154" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -101441,7 +101545,7 @@
         <v>2</v>
       </c>
       <c r="E155" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -101458,7 +101562,7 @@
         <v>2</v>
       </c>
       <c r="E156" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -101475,7 +101579,7 @@
         <v>2</v>
       </c>
       <c r="E157" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -101492,7 +101596,7 @@
         <v>2</v>
       </c>
       <c r="E158" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -101509,7 +101613,7 @@
         <v>2</v>
       </c>
       <c r="E159" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -101526,7 +101630,7 @@
         <v>2</v>
       </c>
       <c r="E160" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -101543,7 +101647,7 @@
         <v>2</v>
       </c>
       <c r="E161" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -101560,7 +101664,7 @@
         <v>2</v>
       </c>
       <c r="E162" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -101577,7 +101681,7 @@
         <v>2</v>
       </c>
       <c r="E163" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -101594,7 +101698,7 @@
         <v>2</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -101611,7 +101715,7 @@
         <v>2</v>
       </c>
       <c r="E165" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -101628,7 +101732,7 @@
         <v>2</v>
       </c>
       <c r="E166" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -101645,7 +101749,7 @@
         <v>2</v>
       </c>
       <c r="E167" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -101662,7 +101766,7 @@
         <v>2</v>
       </c>
       <c r="E168" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -101679,7 +101783,7 @@
         <v>2</v>
       </c>
       <c r="E169" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -101696,7 +101800,7 @@
         <v>2</v>
       </c>
       <c r="E170" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -101713,7 +101817,7 @@
         <v>2</v>
       </c>
       <c r="E171" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -101730,7 +101834,7 @@
         <v>2</v>
       </c>
       <c r="E172" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -101747,7 +101851,7 @@
         <v>2</v>
       </c>
       <c r="E173" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -101764,7 +101868,7 @@
         <v>2</v>
       </c>
       <c r="E174" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -101781,7 +101885,7 @@
         <v>2</v>
       </c>
       <c r="E175" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -101798,7 +101902,7 @@
         <v>2</v>
       </c>
       <c r="E176" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="177" spans="1:5">
@@ -101815,7 +101919,7 @@
         <v>2</v>
       </c>
       <c r="E177" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -101832,7 +101936,7 @@
         <v>1</v>
       </c>
       <c r="E178" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -101849,7 +101953,7 @@
         <v>1</v>
       </c>
       <c r="E179" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -101866,7 +101970,7 @@
         <v>1</v>
       </c>
       <c r="E180" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -101883,7 +101987,7 @@
         <v>1</v>
       </c>
       <c r="E181" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="182" spans="1:5">
@@ -101900,7 +102004,7 @@
         <v>1</v>
       </c>
       <c r="E182" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -101917,7 +102021,7 @@
         <v>1</v>
       </c>
       <c r="E183" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="184" spans="1:5">
@@ -101934,7 +102038,7 @@
         <v>1</v>
       </c>
       <c r="E184" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -101951,7 +102055,7 @@
         <v>1</v>
       </c>
       <c r="E185" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -101968,7 +102072,7 @@
         <v>1</v>
       </c>
       <c r="E186" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="187" spans="1:5">
@@ -101985,7 +102089,7 @@
         <v>1</v>
       </c>
       <c r="E187" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -102002,7 +102106,7 @@
         <v>1</v>
       </c>
       <c r="E188" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -102019,7 +102123,7 @@
         <v>1</v>
       </c>
       <c r="E189" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -102036,7 +102140,7 @@
         <v>1</v>
       </c>
       <c r="E190" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="191" spans="1:5">
@@ -102053,7 +102157,7 @@
         <v>1</v>
       </c>
       <c r="E191" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -102070,7 +102174,7 @@
         <v>1</v>
       </c>
       <c r="E192" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -102087,7 +102191,7 @@
         <v>1</v>
       </c>
       <c r="E193" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -102104,7 +102208,7 @@
         <v>1</v>
       </c>
       <c r="E194" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -102121,7 +102225,7 @@
         <v>1</v>
       </c>
       <c r="E195" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -102138,7 +102242,7 @@
         <v>1</v>
       </c>
       <c r="E196" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -102155,7 +102259,7 @@
         <v>1</v>
       </c>
       <c r="E197" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -102172,7 +102276,7 @@
         <v>1</v>
       </c>
       <c r="E198" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -102189,7 +102293,7 @@
         <v>1</v>
       </c>
       <c r="E199" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -102206,7 +102310,7 @@
         <v>1</v>
       </c>
       <c r="E200" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -102223,7 +102327,7 @@
         <v>1</v>
       </c>
       <c r="E201" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -102240,7 +102344,7 @@
         <v>1</v>
       </c>
       <c r="E202" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -102257,7 +102361,7 @@
         <v>1</v>
       </c>
       <c r="E203" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -102274,7 +102378,7 @@
         <v>1</v>
       </c>
       <c r="E204" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -102291,7 +102395,7 @@
         <v>1</v>
       </c>
       <c r="E205" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -102308,7 +102412,7 @@
         <v>1</v>
       </c>
       <c r="E206" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -102325,7 +102429,7 @@
         <v>1</v>
       </c>
       <c r="E207" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -102342,7 +102446,7 @@
         <v>1</v>
       </c>
       <c r="E208" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -102359,7 +102463,7 @@
         <v>1</v>
       </c>
       <c r="E209" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -102376,7 +102480,7 @@
         <v>1</v>
       </c>
       <c r="E210" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -102393,7 +102497,7 @@
         <v>1</v>
       </c>
       <c r="E211" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -102410,7 +102514,7 @@
         <v>1</v>
       </c>
       <c r="E212" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -102427,7 +102531,7 @@
         <v>1</v>
       </c>
       <c r="E213" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -102444,7 +102548,7 @@
         <v>1</v>
       </c>
       <c r="E214" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -102461,7 +102565,7 @@
         <v>1</v>
       </c>
       <c r="E215" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -102478,7 +102582,7 @@
         <v>1</v>
       </c>
       <c r="E216" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -102495,7 +102599,7 @@
         <v>1</v>
       </c>
       <c r="E217" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -102512,7 +102616,7 @@
         <v>1</v>
       </c>
       <c r="E218" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -102529,7 +102633,7 @@
         <v>1</v>
       </c>
       <c r="E219" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -102546,7 +102650,7 @@
         <v>1</v>
       </c>
       <c r="E220" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -102563,7 +102667,7 @@
         <v>1</v>
       </c>
       <c r="E221" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -102580,7 +102684,7 @@
         <v>1</v>
       </c>
       <c r="E222" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -102597,7 +102701,7 @@
         <v>1</v>
       </c>
       <c r="E223" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -102614,7 +102718,7 @@
         <v>1</v>
       </c>
       <c r="E224" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -102631,7 +102735,7 @@
         <v>2</v>
       </c>
       <c r="E225" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -102648,7 +102752,7 @@
         <v>1</v>
       </c>
       <c r="E226" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -102665,7 +102769,7 @@
         <v>1</v>
       </c>
       <c r="E227" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -102682,7 +102786,7 @@
         <v>1</v>
       </c>
       <c r="E228" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -102699,7 +102803,7 @@
         <v>1</v>
       </c>
       <c r="E229" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -102716,7 +102820,7 @@
         <v>1</v>
       </c>
       <c r="E230" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -102733,7 +102837,7 @@
         <v>1</v>
       </c>
       <c r="E231" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -102750,7 +102854,7 @@
         <v>1</v>
       </c>
       <c r="E232" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -102767,7 +102871,7 @@
         <v>1</v>
       </c>
       <c r="E233" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -102784,7 +102888,7 @@
         <v>1</v>
       </c>
       <c r="E234" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -102801,7 +102905,7 @@
         <v>1</v>
       </c>
       <c r="E235" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -102818,7 +102922,7 @@
         <v>1</v>
       </c>
       <c r="E236" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -102835,7 +102939,7 @@
         <v>1</v>
       </c>
       <c r="E237" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -102852,7 +102956,7 @@
         <v>1</v>
       </c>
       <c r="E238" s="5" t="s">
-        <v>2969</v>
+        <v>2971</v>
       </c>
     </row>
   </sheetData>

</xml_diff>